<commit_message>
thêm execution test suite HTML file cho RECRUIT_VAC execution và toàn bộ code của RECR_VAC
</commit_message>
<xml_diff>
--- a/docs/test-cases/members/Group01_23130299_NguyenVanThang.xlsx
+++ b/docs/test-cases/members/Group01_23130299_NguyenVanThang.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\IdeaProjects\OrangeHRM-Testing\docs\test-cases\members\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4EC5761-3207-479C-8090-CBC40704B205}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C06DDC80-8750-4450-BA57-36138A8AB5FC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="3" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -41,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="968" uniqueCount="692">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="970" uniqueCount="694">
   <si>
     <t>TEST CASE</t>
   </si>
@@ -2615,6 +2615,12 @@
   </si>
   <si>
     <t>M</t>
+  </si>
+  <si>
+    <t>RECRUIT_VAC_20261023_01</t>
+  </si>
+  <si>
+    <t>Katalon Studio / Chrome 155.0.8059.85</t>
   </si>
 </sst>
 </file>
@@ -2820,7 +2826,7 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1"/>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="63">
+  <cellXfs count="64">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
@@ -2931,6 +2937,27 @@
     <xf numFmtId="14" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -2949,14 +2976,6 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -2969,13 +2988,9 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
@@ -2991,13 +3006,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="22" fontId="2" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -3363,14 +3372,14 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:8" ht="42" customHeight="1">
-      <c r="B2" s="44" t="s">
+      <c r="B2" s="38" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="45"/>
-      <c r="D2" s="45"/>
-      <c r="E2" s="45"/>
-      <c r="F2" s="45"/>
-      <c r="G2" s="45"/>
+      <c r="C2" s="39"/>
+      <c r="D2" s="39"/>
+      <c r="E2" s="39"/>
+      <c r="F2" s="39"/>
+      <c r="G2" s="39"/>
       <c r="H2" s="1"/>
     </row>
     <row r="3" spans="2:8">
@@ -3386,11 +3395,11 @@
       <c r="B4" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="46" t="s">
+      <c r="C4" s="40" t="s">
         <v>89</v>
       </c>
-      <c r="D4" s="47"/>
-      <c r="E4" s="47"/>
+      <c r="D4" s="43"/>
+      <c r="E4" s="43"/>
       <c r="F4" s="3" t="s">
         <v>2</v>
       </c>
@@ -3403,11 +3412,11 @@
       <c r="B5" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="46" t="s">
+      <c r="C5" s="40" t="s">
         <v>4</v>
       </c>
-      <c r="D5" s="47"/>
-      <c r="E5" s="47"/>
+      <c r="D5" s="43"/>
+      <c r="E5" s="43"/>
       <c r="F5" s="3" t="s">
         <v>5</v>
       </c>
@@ -3417,14 +3426,14 @@
       <c r="H5" s="1"/>
     </row>
     <row r="6" spans="2:8">
-      <c r="B6" s="48" t="s">
+      <c r="B6" s="53" t="s">
         <v>6</v>
       </c>
-      <c r="C6" s="46" t="s">
+      <c r="C6" s="40" t="s">
         <v>88</v>
       </c>
-      <c r="D6" s="47"/>
-      <c r="E6" s="47"/>
+      <c r="D6" s="43"/>
+      <c r="E6" s="43"/>
       <c r="F6" s="3" t="s">
         <v>7</v>
       </c>
@@ -3434,10 +3443,10 @@
       <c r="H6" s="1"/>
     </row>
     <row r="7" spans="2:8">
-      <c r="B7" s="47"/>
-      <c r="C7" s="47"/>
-      <c r="D7" s="47"/>
-      <c r="E7" s="47"/>
+      <c r="B7" s="43"/>
+      <c r="C7" s="43"/>
+      <c r="D7" s="43"/>
+      <c r="E7" s="43"/>
       <c r="F7" s="3" t="s">
         <v>8</v>
       </c>
@@ -3560,78 +3569,78 @@
       <c r="B16" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="C16" s="49">
+      <c r="C16" s="54">
         <v>23130299</v>
       </c>
-      <c r="D16" s="50"/>
-      <c r="E16" s="50"/>
-      <c r="F16" s="50"/>
-      <c r="G16" s="51"/>
+      <c r="D16" s="55"/>
+      <c r="E16" s="55"/>
+      <c r="F16" s="55"/>
+      <c r="G16" s="56"/>
       <c r="H16" s="1"/>
     </row>
     <row r="17" spans="2:8" ht="24.75" customHeight="1">
       <c r="B17" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="C17" s="38" t="s">
+      <c r="C17" s="47" t="s">
         <v>20</v>
       </c>
-      <c r="D17" s="39"/>
-      <c r="E17" s="39"/>
-      <c r="F17" s="39"/>
-      <c r="G17" s="40"/>
+      <c r="D17" s="48"/>
+      <c r="E17" s="48"/>
+      <c r="F17" s="48"/>
+      <c r="G17" s="49"/>
       <c r="H17" s="1"/>
     </row>
     <row r="18" spans="2:8" ht="24.75" customHeight="1">
       <c r="B18" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="C18" s="38" t="s">
+      <c r="C18" s="47" t="s">
         <v>85</v>
       </c>
-      <c r="D18" s="39"/>
-      <c r="E18" s="39"/>
-      <c r="F18" s="39"/>
-      <c r="G18" s="40"/>
+      <c r="D18" s="48"/>
+      <c r="E18" s="48"/>
+      <c r="F18" s="48"/>
+      <c r="G18" s="49"/>
       <c r="H18" s="1"/>
     </row>
     <row r="19" spans="2:8" ht="24.75" customHeight="1">
       <c r="B19" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="C19" s="38" t="s">
+      <c r="C19" s="47" t="s">
         <v>23</v>
       </c>
-      <c r="D19" s="39"/>
-      <c r="E19" s="39"/>
-      <c r="F19" s="39"/>
-      <c r="G19" s="40"/>
+      <c r="D19" s="48"/>
+      <c r="E19" s="48"/>
+      <c r="F19" s="48"/>
+      <c r="G19" s="49"/>
       <c r="H19" s="1"/>
     </row>
     <row r="20" spans="2:8" ht="36" customHeight="1">
       <c r="B20" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="C20" s="38" t="s">
+      <c r="C20" s="47" t="s">
         <v>651</v>
       </c>
-      <c r="D20" s="39"/>
-      <c r="E20" s="39"/>
-      <c r="F20" s="39"/>
-      <c r="G20" s="40"/>
+      <c r="D20" s="48"/>
+      <c r="E20" s="48"/>
+      <c r="F20" s="48"/>
+      <c r="G20" s="49"/>
       <c r="H20" s="1"/>
     </row>
     <row r="21" spans="2:8" ht="24.75" customHeight="1">
       <c r="B21" s="3" t="s">
         <v>25</v>
       </c>
-      <c r="C21" s="41" t="s">
+      <c r="C21" s="50" t="s">
         <v>90</v>
       </c>
-      <c r="D21" s="42"/>
-      <c r="E21" s="42"/>
-      <c r="F21" s="42"/>
-      <c r="G21" s="43"/>
+      <c r="D21" s="51"/>
+      <c r="E21" s="51"/>
+      <c r="F21" s="51"/>
+      <c r="G21" s="52"/>
       <c r="H21" s="1"/>
     </row>
     <row r="22" spans="2:8" ht="15.75" customHeight="1">
@@ -4656,13 +4665,13 @@
   </cols>
   <sheetData>
     <row r="2" spans="2:8" ht="42" customHeight="1">
-      <c r="B2" s="53" t="s">
+      <c r="B2" s="57" t="s">
         <v>26</v>
       </c>
-      <c r="C2" s="45"/>
-      <c r="D2" s="45"/>
-      <c r="E2" s="45"/>
-      <c r="F2" s="45"/>
+      <c r="C2" s="39"/>
+      <c r="D2" s="39"/>
+      <c r="E2" s="39"/>
+      <c r="F2" s="39"/>
       <c r="G2" s="1"/>
       <c r="H2" s="1"/>
     </row>
@@ -4676,43 +4685,43 @@
       <c r="H3" s="1"/>
     </row>
     <row r="4" spans="2:8">
-      <c r="B4" s="46" t="s">
+      <c r="B4" s="40" t="s">
         <v>1</v>
       </c>
-      <c r="C4" s="54"/>
-      <c r="D4" s="46" t="str">
+      <c r="C4" s="41"/>
+      <c r="D4" s="40" t="str">
         <f>Cover!C4</f>
         <v>OrangeHRM Recruitment</v>
       </c>
-      <c r="E4" s="54"/>
-      <c r="F4" s="54"/>
+      <c r="E4" s="41"/>
+      <c r="F4" s="41"/>
       <c r="G4" s="1"/>
       <c r="H4" s="1"/>
     </row>
     <row r="5" spans="2:8">
-      <c r="B5" s="46" t="s">
+      <c r="B5" s="40" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="54"/>
-      <c r="D5" s="46" t="str">
+      <c r="C5" s="41"/>
+      <c r="D5" s="40" t="str">
         <f>Cover!C5</f>
         <v>Group01_OrangeHRM</v>
       </c>
-      <c r="E5" s="54"/>
-      <c r="F5" s="54"/>
+      <c r="E5" s="41"/>
+      <c r="F5" s="41"/>
       <c r="G5" s="1"/>
       <c r="H5" s="1"/>
     </row>
     <row r="6" spans="2:8" ht="48" customHeight="1">
-      <c r="B6" s="55" t="s">
+      <c r="B6" s="58" t="s">
         <v>27</v>
       </c>
-      <c r="C6" s="54"/>
-      <c r="D6" s="41" t="s">
+      <c r="C6" s="41"/>
+      <c r="D6" s="50" t="s">
         <v>652</v>
       </c>
-      <c r="E6" s="56"/>
-      <c r="F6" s="57"/>
+      <c r="E6" s="59"/>
+      <c r="F6" s="60"/>
       <c r="G6" s="1"/>
       <c r="H6" s="1"/>
     </row>
@@ -4820,11 +4829,11 @@
       <c r="H13" s="1"/>
     </row>
     <row r="14" spans="2:8" ht="37.5" customHeight="1">
-      <c r="B14" s="52"/>
-      <c r="C14" s="45"/>
-      <c r="D14" s="45"/>
-      <c r="E14" s="45"/>
-      <c r="F14" s="45"/>
+      <c r="B14" s="44"/>
+      <c r="C14" s="39"/>
+      <c r="D14" s="39"/>
+      <c r="E14" s="39"/>
+      <c r="F14" s="39"/>
       <c r="G14" s="1"/>
       <c r="H14" s="1"/>
     </row>
@@ -4838,11 +4847,11 @@
       <c r="H15" s="1"/>
     </row>
     <row r="16" spans="2:8" ht="39.75" customHeight="1">
-      <c r="B16" s="52"/>
-      <c r="C16" s="45"/>
-      <c r="D16" s="45"/>
-      <c r="E16" s="45"/>
-      <c r="F16" s="45"/>
+      <c r="B16" s="44"/>
+      <c r="C16" s="39"/>
+      <c r="D16" s="39"/>
+      <c r="E16" s="39"/>
+      <c r="F16" s="39"/>
       <c r="G16" s="1"/>
       <c r="H16" s="1"/>
     </row>
@@ -7254,43 +7263,43 @@
       <c r="A2" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="B2" s="55" t="s">
+      <c r="B2" s="58" t="s">
         <v>94</v>
       </c>
-      <c r="C2" s="54"/>
-      <c r="D2" s="54"/>
-      <c r="E2" s="54"/>
-      <c r="F2" s="54"/>
-      <c r="G2" s="54"/>
-      <c r="H2" s="54"/>
+      <c r="C2" s="41"/>
+      <c r="D2" s="41"/>
+      <c r="E2" s="41"/>
+      <c r="F2" s="41"/>
+      <c r="G2" s="41"/>
+      <c r="H2" s="41"/>
     </row>
     <row r="3" spans="1:8">
       <c r="A3" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="B3" s="55" t="s">
+      <c r="B3" s="58" t="s">
         <v>91</v>
       </c>
-      <c r="C3" s="54"/>
-      <c r="D3" s="54"/>
-      <c r="E3" s="54"/>
-      <c r="F3" s="54"/>
-      <c r="G3" s="54"/>
-      <c r="H3" s="54"/>
+      <c r="C3" s="41"/>
+      <c r="D3" s="41"/>
+      <c r="E3" s="41"/>
+      <c r="F3" s="41"/>
+      <c r="G3" s="41"/>
+      <c r="H3" s="41"/>
     </row>
     <row r="4" spans="1:8">
       <c r="A4" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="B4" s="55" t="s">
+      <c r="B4" s="58" t="s">
         <v>139</v>
       </c>
-      <c r="C4" s="54"/>
-      <c r="D4" s="54"/>
-      <c r="E4" s="54"/>
-      <c r="F4" s="54"/>
-      <c r="G4" s="54"/>
-      <c r="H4" s="54"/>
+      <c r="C4" s="41"/>
+      <c r="D4" s="41"/>
+      <c r="E4" s="41"/>
+      <c r="F4" s="41"/>
+      <c r="G4" s="41"/>
+      <c r="H4" s="41"/>
     </row>
     <row r="5" spans="1:8" ht="24" customHeight="1">
       <c r="A5" s="7" t="s">
@@ -7308,11 +7317,11 @@
       <c r="E5" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="F5" s="58" t="s">
+      <c r="F5" s="61" t="s">
         <v>49</v>
       </c>
-      <c r="G5" s="47"/>
-      <c r="H5" s="47"/>
+      <c r="G5" s="43"/>
+      <c r="H5" s="43"/>
     </row>
     <row r="6" spans="1:8" ht="24" customHeight="1">
       <c r="A6" s="8">
@@ -7335,12 +7344,12 @@
         <f>COUNTIF($F$9:$F$33,"Skipped")</f>
         <v>0</v>
       </c>
-      <c r="F6" s="59">
+      <c r="F6" s="62">
         <f>COUNTA(A9:A33)</f>
         <v>25</v>
       </c>
-      <c r="G6" s="54"/>
-      <c r="H6" s="54"/>
+      <c r="G6" s="41"/>
+      <c r="H6" s="41"/>
     </row>
     <row r="7" spans="1:8">
       <c r="A7" s="1"/>
@@ -9059,43 +9068,43 @@
       <c r="A2" s="23" t="s">
         <v>41</v>
       </c>
-      <c r="B2" s="43" t="s">
+      <c r="B2" s="52" t="s">
         <v>114</v>
       </c>
-      <c r="C2" s="54"/>
-      <c r="D2" s="54"/>
-      <c r="E2" s="54"/>
-      <c r="F2" s="54"/>
-      <c r="G2" s="54"/>
-      <c r="H2" s="54"/>
+      <c r="C2" s="41"/>
+      <c r="D2" s="41"/>
+      <c r="E2" s="41"/>
+      <c r="F2" s="41"/>
+      <c r="G2" s="41"/>
+      <c r="H2" s="41"/>
     </row>
     <row r="3" spans="1:8">
       <c r="A3" s="23" t="s">
         <v>42</v>
       </c>
-      <c r="B3" s="43" t="s">
+      <c r="B3" s="52" t="s">
         <v>92</v>
       </c>
-      <c r="C3" s="54"/>
-      <c r="D3" s="54"/>
-      <c r="E3" s="54"/>
-      <c r="F3" s="54"/>
-      <c r="G3" s="54"/>
-      <c r="H3" s="54"/>
+      <c r="C3" s="41"/>
+      <c r="D3" s="41"/>
+      <c r="E3" s="41"/>
+      <c r="F3" s="41"/>
+      <c r="G3" s="41"/>
+      <c r="H3" s="41"/>
     </row>
     <row r="4" spans="1:8">
       <c r="A4" s="23" t="s">
         <v>43</v>
       </c>
-      <c r="B4" s="43" t="s">
+      <c r="B4" s="52" t="s">
         <v>139</v>
       </c>
-      <c r="C4" s="54"/>
-      <c r="D4" s="54"/>
-      <c r="E4" s="54"/>
-      <c r="F4" s="54"/>
-      <c r="G4" s="54"/>
-      <c r="H4" s="54"/>
+      <c r="C4" s="41"/>
+      <c r="D4" s="41"/>
+      <c r="E4" s="41"/>
+      <c r="F4" s="41"/>
+      <c r="G4" s="41"/>
+      <c r="H4" s="41"/>
     </row>
     <row r="5" spans="1:8" ht="24" customHeight="1">
       <c r="A5" s="24" t="s">
@@ -9113,11 +9122,11 @@
       <c r="E5" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="F5" s="58" t="s">
+      <c r="F5" s="61" t="s">
         <v>49</v>
       </c>
-      <c r="G5" s="47"/>
-      <c r="H5" s="47"/>
+      <c r="G5" s="43"/>
+      <c r="H5" s="43"/>
     </row>
     <row r="6" spans="1:8" ht="24" customHeight="1">
       <c r="A6" s="25">
@@ -9140,12 +9149,12 @@
         <f>COUNTIF($F$9:$F$33,"Skipped")</f>
         <v>0</v>
       </c>
-      <c r="F6" s="59">
+      <c r="F6" s="62">
         <f>COUNTA(A9:A33)</f>
         <v>25</v>
       </c>
-      <c r="G6" s="54"/>
-      <c r="H6" s="54"/>
+      <c r="G6" s="41"/>
+      <c r="H6" s="41"/>
     </row>
     <row r="7" spans="1:8">
       <c r="A7" s="29"/>
@@ -10814,43 +10823,43 @@
       <c r="A2" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="B2" s="55" t="s">
+      <c r="B2" s="58" t="s">
         <v>126</v>
       </c>
-      <c r="C2" s="54"/>
-      <c r="D2" s="54"/>
-      <c r="E2" s="54"/>
-      <c r="F2" s="54"/>
-      <c r="G2" s="54"/>
-      <c r="H2" s="54"/>
+      <c r="C2" s="41"/>
+      <c r="D2" s="41"/>
+      <c r="E2" s="41"/>
+      <c r="F2" s="41"/>
+      <c r="G2" s="41"/>
+      <c r="H2" s="41"/>
     </row>
     <row r="3" spans="1:8">
       <c r="A3" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="B3" s="55" t="s">
+      <c r="B3" s="58" t="s">
         <v>93</v>
       </c>
-      <c r="C3" s="54"/>
-      <c r="D3" s="54"/>
-      <c r="E3" s="54"/>
-      <c r="F3" s="54"/>
-      <c r="G3" s="54"/>
-      <c r="H3" s="54"/>
+      <c r="C3" s="41"/>
+      <c r="D3" s="41"/>
+      <c r="E3" s="41"/>
+      <c r="F3" s="41"/>
+      <c r="G3" s="41"/>
+      <c r="H3" s="41"/>
     </row>
     <row r="4" spans="1:8">
       <c r="A4" s="3" t="s">
         <v>43</v>
       </c>
-      <c r="B4" s="43" t="s">
+      <c r="B4" s="52" t="s">
         <v>139</v>
       </c>
-      <c r="C4" s="54"/>
-      <c r="D4" s="54"/>
-      <c r="E4" s="54"/>
-      <c r="F4" s="54"/>
-      <c r="G4" s="54"/>
-      <c r="H4" s="54"/>
+      <c r="C4" s="41"/>
+      <c r="D4" s="41"/>
+      <c r="E4" s="41"/>
+      <c r="F4" s="41"/>
+      <c r="G4" s="41"/>
+      <c r="H4" s="41"/>
     </row>
     <row r="5" spans="1:8" ht="24" customHeight="1">
       <c r="A5" s="7" t="s">
@@ -10868,11 +10877,11 @@
       <c r="E5" s="7" t="s">
         <v>48</v>
       </c>
-      <c r="F5" s="58" t="s">
+      <c r="F5" s="61" t="s">
         <v>49</v>
       </c>
-      <c r="G5" s="47"/>
-      <c r="H5" s="47"/>
+      <c r="G5" s="43"/>
+      <c r="H5" s="43"/>
     </row>
     <row r="6" spans="1:8" ht="24" customHeight="1">
       <c r="A6" s="8">
@@ -10895,12 +10904,12 @@
         <f>COUNTIF($F$9:$F$33,"Skipped")</f>
         <v>0</v>
       </c>
-      <c r="F6" s="59">
+      <c r="F6" s="62">
         <f>COUNTA(A9:A33)</f>
         <v>25</v>
       </c>
-      <c r="G6" s="54"/>
-      <c r="H6" s="54"/>
+      <c r="G6" s="41"/>
+      <c r="H6" s="41"/>
     </row>
     <row r="7" spans="1:8">
       <c r="A7" s="1"/>
@@ -12559,14 +12568,14 @@
       <c r="F1" s="1"/>
     </row>
     <row r="2" spans="1:6" ht="42" customHeight="1">
-      <c r="A2" s="53" t="s">
+      <c r="A2" s="57" t="s">
         <v>367</v>
       </c>
-      <c r="B2" s="45"/>
-      <c r="C2" s="45"/>
-      <c r="D2" s="45"/>
-      <c r="E2" s="45"/>
-      <c r="F2" s="45"/>
+      <c r="B2" s="39"/>
+      <c r="C2" s="39"/>
+      <c r="D2" s="39"/>
+      <c r="E2" s="39"/>
+      <c r="F2" s="39"/>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" s="1"/>
@@ -14024,14 +14033,14 @@
       <c r="F1" s="1"/>
     </row>
     <row r="2" spans="1:6" ht="42" customHeight="1">
-      <c r="A2" s="44" t="s">
+      <c r="A2" s="38" t="s">
         <v>70</v>
       </c>
-      <c r="B2" s="45"/>
-      <c r="C2" s="45"/>
-      <c r="D2" s="45"/>
-      <c r="E2" s="45"/>
-      <c r="F2" s="45"/>
+      <c r="B2" s="39"/>
+      <c r="C2" s="39"/>
+      <c r="D2" s="39"/>
+      <c r="E2" s="39"/>
+      <c r="F2" s="39"/>
     </row>
     <row r="3" spans="1:6">
       <c r="A3" s="1"/>
@@ -15354,16 +15363,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="2:9" ht="42" customHeight="1">
-      <c r="B1" s="44" t="s">
+      <c r="B1" s="38" t="s">
         <v>76</v>
       </c>
-      <c r="C1" s="45"/>
-      <c r="D1" s="45"/>
-      <c r="E1" s="45"/>
-      <c r="F1" s="45"/>
-      <c r="G1" s="45"/>
-      <c r="H1" s="45"/>
-      <c r="I1" s="45"/>
+      <c r="C1" s="39"/>
+      <c r="D1" s="39"/>
+      <c r="E1" s="39"/>
+      <c r="F1" s="39"/>
+      <c r="G1" s="39"/>
+      <c r="H1" s="39"/>
+      <c r="I1" s="39"/>
     </row>
     <row r="2" spans="2:9">
       <c r="B2" s="1"/>
@@ -15376,58 +15385,64 @@
       <c r="I2" s="1"/>
     </row>
     <row r="3" spans="2:9">
-      <c r="B3" s="46" t="s">
+      <c r="B3" s="40" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="54"/>
-      <c r="D3" s="46" t="str">
+      <c r="C3" s="41"/>
+      <c r="D3" s="40" t="str">
         <f>Cover!C4</f>
         <v>OrangeHRM Recruitment</v>
       </c>
-      <c r="E3" s="54"/>
-      <c r="F3" s="54"/>
-      <c r="G3" s="54"/>
-      <c r="H3" s="54"/>
-      <c r="I3" s="54"/>
+      <c r="E3" s="41"/>
+      <c r="F3" s="41"/>
+      <c r="G3" s="41"/>
+      <c r="H3" s="41"/>
+      <c r="I3" s="41"/>
     </row>
     <row r="4" spans="2:9">
-      <c r="B4" s="46" t="s">
+      <c r="B4" s="40" t="s">
         <v>6</v>
       </c>
-      <c r="C4" s="54"/>
-      <c r="D4" s="46" t="str">
+      <c r="C4" s="41"/>
+      <c r="D4" s="40" t="str">
         <f>Cover!C6</f>
         <v>Group01_23130299_NguyenVanThang</v>
       </c>
-      <c r="E4" s="54"/>
-      <c r="F4" s="54"/>
-      <c r="G4" s="54"/>
-      <c r="H4" s="54"/>
-      <c r="I4" s="54"/>
+      <c r="E4" s="41"/>
+      <c r="F4" s="41"/>
+      <c r="G4" s="41"/>
+      <c r="H4" s="41"/>
+      <c r="I4" s="41"/>
     </row>
     <row r="5" spans="2:9">
-      <c r="B5" s="46" t="s">
+      <c r="B5" s="40" t="s">
         <v>77</v>
       </c>
-      <c r="C5" s="54"/>
-      <c r="D5" s="60"/>
-      <c r="E5" s="47"/>
-      <c r="F5" s="47"/>
-      <c r="G5" s="60"/>
-      <c r="H5" s="47"/>
-      <c r="I5" s="47"/>
+      <c r="C5" s="41"/>
+      <c r="D5" s="42" t="s">
+        <v>692</v>
+      </c>
+      <c r="E5" s="43"/>
+      <c r="F5" s="43"/>
+      <c r="G5" s="63">
+        <v>46318.496458333335</v>
+      </c>
+      <c r="H5" s="43"/>
+      <c r="I5" s="43"/>
     </row>
     <row r="6" spans="2:9">
-      <c r="B6" s="46" t="s">
+      <c r="B6" s="40" t="s">
         <v>78</v>
       </c>
-      <c r="C6" s="54"/>
-      <c r="D6" s="60"/>
-      <c r="E6" s="47"/>
-      <c r="F6" s="47"/>
-      <c r="G6" s="47"/>
-      <c r="H6" s="47"/>
-      <c r="I6" s="47"/>
+      <c r="C6" s="41"/>
+      <c r="D6" s="42" t="s">
+        <v>693</v>
+      </c>
+      <c r="E6" s="43"/>
+      <c r="F6" s="43"/>
+      <c r="G6" s="43"/>
+      <c r="H6" s="43"/>
+      <c r="I6" s="43"/>
     </row>
     <row r="7" spans="2:9">
       <c r="B7" s="1"/>
@@ -15582,10 +15597,10 @@
       <c r="I13" s="1"/>
     </row>
     <row r="14" spans="2:9">
-      <c r="B14" s="61" t="s">
+      <c r="B14" s="45" t="s">
         <v>79</v>
       </c>
-      <c r="C14" s="47"/>
+      <c r="C14" s="43"/>
       <c r="D14" s="13">
         <f t="shared" ref="D14:I14" si="0">SUM(D10:D12)</f>
         <v>23</v>
@@ -15632,31 +15647,31 @@
       <c r="I16" s="1"/>
     </row>
     <row r="17" spans="2:9">
-      <c r="B17" s="46" t="s">
+      <c r="B17" s="40" t="s">
         <v>80</v>
       </c>
-      <c r="C17" s="54"/>
-      <c r="D17" s="54"/>
-      <c r="E17" s="62">
+      <c r="C17" s="41"/>
+      <c r="D17" s="41"/>
+      <c r="E17" s="46">
         <f>IF(I14=0,"",(D14+E14)/I14)</f>
         <v>0.33333333333333331</v>
       </c>
-      <c r="F17" s="54"/>
+      <c r="F17" s="41"/>
       <c r="G17" s="1"/>
       <c r="H17" s="1"/>
       <c r="I17" s="1"/>
     </row>
     <row r="18" spans="2:9">
-      <c r="B18" s="46" t="s">
+      <c r="B18" s="40" t="s">
         <v>81</v>
       </c>
-      <c r="C18" s="54"/>
-      <c r="D18" s="54"/>
-      <c r="E18" s="62">
+      <c r="C18" s="41"/>
+      <c r="D18" s="41"/>
+      <c r="E18" s="46">
         <f>IF(D14+E14=0,"Chưa thực thi",D14/(D14+E14))</f>
         <v>0.92</v>
       </c>
-      <c r="F18" s="54"/>
+      <c r="F18" s="41"/>
       <c r="G18" s="1"/>
       <c r="H18" s="1"/>
       <c r="I18" s="1"/>
@@ -15672,16 +15687,16 @@
       <c r="I19" s="1"/>
     </row>
     <row r="20" spans="2:9" ht="39.75" customHeight="1">
-      <c r="B20" s="52" t="s">
+      <c r="B20" s="44" t="s">
         <v>82</v>
       </c>
-      <c r="C20" s="45"/>
-      <c r="D20" s="45"/>
-      <c r="E20" s="45"/>
-      <c r="F20" s="45"/>
-      <c r="G20" s="45"/>
-      <c r="H20" s="45"/>
-      <c r="I20" s="45"/>
+      <c r="C20" s="39"/>
+      <c r="D20" s="39"/>
+      <c r="E20" s="39"/>
+      <c r="F20" s="39"/>
+      <c r="G20" s="39"/>
+      <c r="H20" s="39"/>
+      <c r="I20" s="39"/>
     </row>
     <row r="21" spans="2:9" ht="15.75" customHeight="1">
       <c r="B21" s="1"/>
@@ -15694,16 +15709,16 @@
       <c r="I21" s="1"/>
     </row>
     <row r="22" spans="2:9" ht="39.75" customHeight="1">
-      <c r="B22" s="52" t="s">
+      <c r="B22" s="44" t="s">
         <v>83</v>
       </c>
-      <c r="C22" s="45"/>
-      <c r="D22" s="45"/>
-      <c r="E22" s="45"/>
-      <c r="F22" s="45"/>
-      <c r="G22" s="45"/>
-      <c r="H22" s="45"/>
-      <c r="I22" s="45"/>
+      <c r="C22" s="39"/>
+      <c r="D22" s="39"/>
+      <c r="E22" s="39"/>
+      <c r="F22" s="39"/>
+      <c r="G22" s="39"/>
+      <c r="H22" s="39"/>
+      <c r="I22" s="39"/>
     </row>
     <row r="23" spans="2:9" ht="15.75" customHeight="1">
       <c r="B23" s="1"/>
@@ -16694,11 +16709,6 @@
     <row r="1000" ht="15.75" customHeight="1"/>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="B1:I1"/>
-    <mergeCell ref="B3:C3"/>
-    <mergeCell ref="D3:I3"/>
-    <mergeCell ref="B4:C4"/>
-    <mergeCell ref="D4:I4"/>
     <mergeCell ref="D5:F5"/>
     <mergeCell ref="G5:I5"/>
     <mergeCell ref="D6:I6"/>
@@ -16711,6 +16721,11 @@
     <mergeCell ref="E17:F17"/>
     <mergeCell ref="B18:D18"/>
     <mergeCell ref="E18:F18"/>
+    <mergeCell ref="B1:I1"/>
+    <mergeCell ref="B3:C3"/>
+    <mergeCell ref="D3:I3"/>
+    <mergeCell ref="B4:C4"/>
+    <mergeCell ref="D4:I4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>